<commit_message>
Work 25 June v1
</commit_message>
<xml_diff>
--- a/AtchisonRegime/Outputs/Aust/ASX300/df_TESTCONTOUR_grouped.xlsx
+++ b/AtchisonRegime/Outputs/Aust/ASX300/df_TESTCONTOUR_grouped.xlsx
@@ -1506,7 +1506,7 @@
         <v>0.2</v>
       </c>
       <c r="D77" t="n">
-        <v>1.645157026629973</v>
+        <v>7.516578634510473</v>
       </c>
     </row>
     <row r="78">
@@ -4492,13 +4492,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A8A49170-7497-4AF2-A37B-1CBF0721F55F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DD21361-6F01-4EF7-8A16-0B5C029399E6}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0B2A2B63-762F-4D11-ADE5-31BADA6A7DAD}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1C1D2A0A-90E0-419B-B7FE-239A8A8E7A79}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA304D75-DD1A-46A4-AB9C-F4076D4281E7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C6D4B26A-7DBF-4BEC-A7F2-0B2CD0D325F8}"/>
 </file>
</xml_diff>